<commit_message>
introduce the vg pack 1.7
</commit_message>
<xml_diff>
--- a/VEEPortingGuide/ui_vg_releases_notes_cco.xlsx
+++ b/VEEPortingGuide/ui_vg_releases_notes_cco.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git_pub\docs\VEEPortingGuide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4656DD8-2D0A-4437-BDD2-A872760A7190}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04DC6B09-22D2-4673-9622-B97394F04EC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="502" xr2:uid="{62F6EEB7-C17F-40C9-8050-F3352CC93ED9}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="94">
   <si>
     <t>pack ui</t>
   </si>
@@ -311,6 +311,9 @@
   </si>
   <si>
     <t>10.0.0</t>
+  </si>
+  <si>
+    <t>1.7.0</t>
   </si>
 </sst>
 </file>
@@ -1106,7 +1109,9 @@
         <v>92</v>
       </c>
       <c r="E14" s="1"/>
-      <c r="H14" s="10"/>
+      <c r="H14" s="11" t="s">
+        <v>93</v>
+      </c>
       <c r="I14" s="1"/>
       <c r="J14" s="11" t="s">
         <v>7</v>
@@ -1292,7 +1297,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E750B59-6D36-4DC3-86F9-7C4DB63A361C}">
-  <dimension ref="A1:AS179"/>
+  <dimension ref="A1:AS181"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.140625" style="1" bestFit="1" customWidth="1"/>
@@ -18321,67 +18326,67 @@
         <v/>
       </c>
       <c r="AC133" s="1" t="str">
-        <f t="shared" ref="AC133:AC179" si="65">IF($I133=0,"",$G133)</f>
+        <f t="shared" ref="AC133:AC181" si="65">IF($I133=0,"",$G133)</f>
         <v>1.4.0</v>
       </c>
       <c r="AD133" s="1" t="str">
-        <f t="shared" ref="AD133:AD179" si="66">IF($I133=0,"",$A133)</f>
+        <f t="shared" ref="AD133:AD181" si="66">IF($I133=0,"",$A133)</f>
         <v>13.7.2</v>
       </c>
       <c r="AE133" s="1" t="str">
-        <f t="shared" ref="AE133:AE179" si="67">IF($I133=0,"",$I133)</f>
+        <f t="shared" ref="AE133:AE181" si="67">IF($I133=0,"",$I133)</f>
         <v>6.0.0</v>
       </c>
       <c r="AF133" s="1" t="str">
-        <f t="shared" ref="AF133:AF179" si="68">IF($I133=0,"",$D133)</f>
+        <f t="shared" ref="AF133:AF181" si="68">IF($I133=0,"",$D133)</f>
         <v>7.2.0</v>
       </c>
       <c r="AG133" s="1" t="str">
-        <f t="shared" ref="AG133:AG179" si="69">IF($I133=0,"",$H133)</f>
+        <f t="shared" ref="AG133:AG181" si="69">IF($I133=0,"",$H133)</f>
         <v>3.0.1</v>
       </c>
       <c r="AH133" s="1" t="str">
-        <f t="shared" ref="AH133:AH179" si="70">IF($I133=0,"",$B133)</f>
+        <f t="shared" ref="AH133:AH181" si="70">IF($I133=0,"",$B133)</f>
         <v>3.1.0</v>
       </c>
       <c r="AI133" s="1" t="str">
-        <f t="shared" ref="AI133:AI179" si="71">IF($I133=0,"",$K133)</f>
+        <f t="shared" ref="AI133:AI181" si="71">IF($I133=0,"",$K133)</f>
         <v>2.0.2</v>
       </c>
       <c r="AJ133" s="1" t="str">
-        <f t="shared" ref="AJ133:AJ179" si="72">IF($I133=0,"",$L133)</f>
+        <f t="shared" ref="AJ133:AJ181" si="72">IF($I133=0,"",$L133)</f>
         <v>1.0.2</v>
       </c>
       <c r="AL133" s="1" t="str">
-        <f t="shared" ref="AL133:AL179" si="73">IF($J133=0,"",$G133)</f>
+        <f t="shared" ref="AL133:AL181" si="73">IF($J133=0,"",$G133)</f>
         <v/>
       </c>
       <c r="AM133" s="1" t="str">
-        <f t="shared" ref="AM133:AM179" si="74">IF($J133=0,"",$A133)</f>
+        <f t="shared" ref="AM133:AM181" si="74">IF($J133=0,"",$A133)</f>
         <v/>
       </c>
       <c r="AN133" s="1" t="str">
-        <f t="shared" ref="AN133:AN179" si="75">IF($J133=0,"",$J133)</f>
+        <f t="shared" ref="AN133:AN181" si="75">IF($J133=0,"",$J133)</f>
         <v/>
       </c>
       <c r="AO133" s="1" t="str">
-        <f t="shared" ref="AO133:AO179" si="76">IF($J133=0,"",$E133)</f>
+        <f t="shared" ref="AO133:AO181" si="76">IF($J133=0,"",$E133)</f>
         <v/>
       </c>
       <c r="AP133" s="1" t="str">
-        <f t="shared" ref="AP133:AP179" si="77">IF($J133=0,"",$H133)</f>
+        <f t="shared" ref="AP133:AP181" si="77">IF($J133=0,"",$H133)</f>
         <v/>
       </c>
       <c r="AQ133" s="1" t="str">
-        <f t="shared" ref="AQ133:AQ179" si="78">IF($J133=0,"",$B133)</f>
+        <f t="shared" ref="AQ133:AQ181" si="78">IF($J133=0,"",$B133)</f>
         <v/>
       </c>
       <c r="AR133" s="1" t="str">
-        <f t="shared" ref="AR133:AR179" si="79">IF($J133=0,"",$K133)</f>
+        <f t="shared" ref="AR133:AR181" si="79">IF($J133=0,"",$K133)</f>
         <v/>
       </c>
       <c r="AS133" s="1" t="str">
-        <f t="shared" ref="AS133:AS179" si="80">IF($J133=0,"",$L133)</f>
+        <f t="shared" ref="AS133:AS181" si="80">IF($J133=0,"",$L133)</f>
         <v/>
       </c>
     </row>
@@ -23532,7 +23537,7 @@
         <v>14.1.0</v>
       </c>
       <c r="B173" s="3" t="str">
-        <f t="shared" ref="B173:B179" si="128">A173</f>
+        <f t="shared" ref="B173:B181" si="128">A173</f>
         <v>14.1.0</v>
       </c>
       <c r="C173" s="3" t="s">
@@ -24346,21 +24351,21 @@
         <v>14.1.0</v>
       </c>
       <c r="C179" s="3"/>
-      <c r="D179" s="12"/>
-      <c r="E179" s="12" t="s">
-        <v>31</v>
-      </c>
+      <c r="D179" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="E179" s="12"/>
       <c r="F179" s="12"/>
       <c r="G179" s="12" t="s">
-        <v>47</v>
+        <v>93</v>
       </c>
       <c r="H179" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="I179" s="12"/>
-      <c r="J179" s="12" t="s">
-        <v>49</v>
-      </c>
+      <c r="I179" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="J179" s="12"/>
       <c r="K179" s="12" t="s">
         <v>29</v>
       </c>
@@ -24368,110 +24373,390 @@
         <v>49</v>
       </c>
       <c r="N179" s="1" t="str">
-        <f t="shared" si="117"/>
+        <f t="shared" ref="N179" si="131">A179</f>
         <v>14.1.0</v>
       </c>
       <c r="O179" s="1" t="str">
-        <f t="shared" si="118"/>
+        <f t="shared" ref="O179" si="132">B179</f>
         <v>14.1.0</v>
       </c>
       <c r="Q179" s="1" t="str">
-        <f t="shared" si="119"/>
+        <f t="shared" ref="Q179" si="133">IF(C179=0,"",$A179)</f>
         <v/>
       </c>
       <c r="R179" s="1" t="str">
-        <f t="shared" si="120"/>
+        <f t="shared" ref="R179" si="134">IF(C179=0,"",$C179)</f>
         <v/>
       </c>
       <c r="S179" s="1" t="str">
-        <f t="shared" si="121"/>
+        <f t="shared" ref="S179" si="135">IF(C179=0,"",$B179)</f>
         <v/>
       </c>
       <c r="U179" s="1" t="str">
-        <f t="shared" si="122"/>
-        <v/>
+        <f t="shared" ref="U179" si="136">IF(D179=0,"",$A179)</f>
+        <v>14.1.0</v>
       </c>
       <c r="V179" s="1" t="str">
-        <f t="shared" si="123"/>
-        <v/>
+        <f t="shared" ref="V179" si="137">IF(D179=0,"",$D179)</f>
+        <v>10.0.0</v>
       </c>
       <c r="W179" s="1" t="str">
-        <f t="shared" si="124"/>
-        <v/>
+        <f t="shared" ref="W179" si="138">IF(D179=0,"",$B179)</f>
+        <v>14.1.0</v>
       </c>
       <c r="Y179" s="1" t="str">
-        <f t="shared" si="125"/>
-        <v>14.1.0</v>
+        <f t="shared" ref="Y179" si="139">IF(E179=0,"",$A179)</f>
+        <v/>
       </c>
       <c r="Z179" s="1" t="str">
-        <f t="shared" si="126"/>
-        <v>4.0.0</v>
+        <f t="shared" ref="Z179" si="140">IF(E179=0,"",$E179)</f>
+        <v/>
       </c>
       <c r="AA179" s="1" t="str">
-        <f t="shared" si="127"/>
-        <v>14.1.0</v>
+        <f t="shared" ref="AA179" si="141">IF(E179=0,"",$B179)</f>
+        <v/>
       </c>
       <c r="AC179" s="1" t="str">
         <f t="shared" si="65"/>
-        <v/>
+        <v>1.7.0</v>
       </c>
       <c r="AD179" s="1" t="str">
         <f t="shared" si="66"/>
-        <v/>
+        <v>14.1.0</v>
       </c>
       <c r="AE179" s="1" t="str">
         <f t="shared" si="67"/>
-        <v/>
+        <v>9.0.0</v>
       </c>
       <c r="AF179" s="1" t="str">
         <f t="shared" si="68"/>
-        <v/>
+        <v>10.0.0</v>
       </c>
       <c r="AG179" s="1" t="str">
         <f t="shared" si="69"/>
-        <v/>
+        <v>7.0.0</v>
       </c>
       <c r="AH179" s="1" t="str">
         <f t="shared" si="70"/>
-        <v/>
+        <v>14.1.0</v>
       </c>
       <c r="AI179" s="1" t="str">
         <f t="shared" si="71"/>
-        <v/>
+        <v>3.0.0</v>
       </c>
       <c r="AJ179" s="1" t="str">
         <f t="shared" si="72"/>
-        <v/>
+        <v>2.0.0</v>
       </c>
       <c r="AL179" s="1" t="str">
         <f t="shared" si="73"/>
-        <v>1.6.0</v>
+        <v/>
       </c>
       <c r="AM179" s="1" t="str">
         <f t="shared" si="74"/>
-        <v>14.1.0</v>
+        <v/>
       </c>
       <c r="AN179" s="1" t="str">
         <f t="shared" si="75"/>
-        <v>2.0.0</v>
+        <v/>
       </c>
       <c r="AO179" s="1" t="str">
         <f t="shared" si="76"/>
-        <v>4.0.0</v>
+        <v/>
       </c>
       <c r="AP179" s="1" t="str">
         <f t="shared" si="77"/>
-        <v>7.0.0</v>
+        <v/>
       </c>
       <c r="AQ179" s="1" t="str">
         <f t="shared" si="78"/>
-        <v>14.1.0</v>
+        <v/>
       </c>
       <c r="AR179" s="1" t="str">
         <f t="shared" si="79"/>
+        <v/>
+      </c>
+      <c r="AS179" s="1" t="str">
+        <f t="shared" si="80"/>
+        <v/>
+      </c>
+    </row>
+    <row r="180" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A180" s="3" t="str">
+        <f t="shared" ref="A180" si="142">A179</f>
+        <v>14.1.0</v>
+      </c>
+      <c r="B180" s="3" t="str">
+        <f t="shared" si="128"/>
+        <v>14.1.0</v>
+      </c>
+      <c r="C180" s="3"/>
+      <c r="D180" s="12"/>
+      <c r="E180" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F180" s="12"/>
+      <c r="G180" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="H180" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="I180" s="12"/>
+      <c r="J180" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="K180" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="L180" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="N180" s="1" t="str">
+        <f t="shared" ref="N180" si="143">A180</f>
+        <v>14.1.0</v>
+      </c>
+      <c r="O180" s="1" t="str">
+        <f t="shared" ref="O180" si="144">B180</f>
+        <v>14.1.0</v>
+      </c>
+      <c r="Q180" s="1" t="str">
+        <f t="shared" ref="Q180" si="145">IF(C180=0,"",$A180)</f>
+        <v/>
+      </c>
+      <c r="R180" s="1" t="str">
+        <f t="shared" ref="R180" si="146">IF(C180=0,"",$C180)</f>
+        <v/>
+      </c>
+      <c r="S180" s="1" t="str">
+        <f t="shared" ref="S180" si="147">IF(C180=0,"",$B180)</f>
+        <v/>
+      </c>
+      <c r="U180" s="1" t="str">
+        <f t="shared" ref="U180" si="148">IF(D180=0,"",$A180)</f>
+        <v/>
+      </c>
+      <c r="V180" s="1" t="str">
+        <f t="shared" ref="V180" si="149">IF(D180=0,"",$D180)</f>
+        <v/>
+      </c>
+      <c r="W180" s="1" t="str">
+        <f t="shared" ref="W180" si="150">IF(D180=0,"",$B180)</f>
+        <v/>
+      </c>
+      <c r="Y180" s="1" t="str">
+        <f t="shared" ref="Y180" si="151">IF(E180=0,"",$A180)</f>
+        <v>14.1.0</v>
+      </c>
+      <c r="Z180" s="1" t="str">
+        <f t="shared" ref="Z180" si="152">IF(E180=0,"",$E180)</f>
+        <v>4.0.0</v>
+      </c>
+      <c r="AA180" s="1" t="str">
+        <f t="shared" ref="AA180" si="153">IF(E180=0,"",$B180)</f>
+        <v>14.1.0</v>
+      </c>
+      <c r="AC180" s="1" t="str">
+        <f t="shared" si="65"/>
+        <v/>
+      </c>
+      <c r="AD180" s="1" t="str">
+        <f t="shared" si="66"/>
+        <v/>
+      </c>
+      <c r="AE180" s="1" t="str">
+        <f t="shared" si="67"/>
+        <v/>
+      </c>
+      <c r="AF180" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v/>
+      </c>
+      <c r="AG180" s="1" t="str">
+        <f t="shared" si="69"/>
+        <v/>
+      </c>
+      <c r="AH180" s="1" t="str">
+        <f t="shared" si="70"/>
+        <v/>
+      </c>
+      <c r="AI180" s="1" t="str">
+        <f t="shared" si="71"/>
+        <v/>
+      </c>
+      <c r="AJ180" s="1" t="str">
+        <f t="shared" si="72"/>
+        <v/>
+      </c>
+      <c r="AL180" s="1" t="str">
+        <f t="shared" si="73"/>
+        <v>1.6.0</v>
+      </c>
+      <c r="AM180" s="1" t="str">
+        <f t="shared" si="74"/>
+        <v>14.1.0</v>
+      </c>
+      <c r="AN180" s="1" t="str">
+        <f t="shared" si="75"/>
+        <v>2.0.0</v>
+      </c>
+      <c r="AO180" s="1" t="str">
+        <f t="shared" si="76"/>
+        <v>4.0.0</v>
+      </c>
+      <c r="AP180" s="1" t="str">
+        <f t="shared" si="77"/>
+        <v>7.0.0</v>
+      </c>
+      <c r="AQ180" s="1" t="str">
+        <f t="shared" si="78"/>
+        <v>14.1.0</v>
+      </c>
+      <c r="AR180" s="1" t="str">
+        <f t="shared" si="79"/>
         <v>3.0.0</v>
       </c>
-      <c r="AS179" s="1" t="str">
+      <c r="AS180" s="1" t="str">
+        <f t="shared" si="80"/>
+        <v>2.0.0</v>
+      </c>
+    </row>
+    <row r="181" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A181" s="3" t="str">
+        <f t="shared" ref="A181" si="154">A180</f>
+        <v>14.1.0</v>
+      </c>
+      <c r="B181" s="3" t="str">
+        <f t="shared" si="128"/>
+        <v>14.1.0</v>
+      </c>
+      <c r="C181" s="3"/>
+      <c r="D181" s="12"/>
+      <c r="E181" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F181" s="12"/>
+      <c r="G181" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="H181" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="I181" s="12"/>
+      <c r="J181" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="K181" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="L181" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="N181" s="1" t="str">
+        <f t="shared" ref="N181" si="155">A181</f>
+        <v>14.1.0</v>
+      </c>
+      <c r="O181" s="1" t="str">
+        <f t="shared" ref="O181" si="156">B181</f>
+        <v>14.1.0</v>
+      </c>
+      <c r="Q181" s="1" t="str">
+        <f t="shared" ref="Q181" si="157">IF(C181=0,"",$A181)</f>
+        <v/>
+      </c>
+      <c r="R181" s="1" t="str">
+        <f t="shared" ref="R181" si="158">IF(C181=0,"",$C181)</f>
+        <v/>
+      </c>
+      <c r="S181" s="1" t="str">
+        <f t="shared" ref="S181" si="159">IF(C181=0,"",$B181)</f>
+        <v/>
+      </c>
+      <c r="U181" s="1" t="str">
+        <f t="shared" ref="U181" si="160">IF(D181=0,"",$A181)</f>
+        <v/>
+      </c>
+      <c r="V181" s="1" t="str">
+        <f t="shared" ref="V181" si="161">IF(D181=0,"",$D181)</f>
+        <v/>
+      </c>
+      <c r="W181" s="1" t="str">
+        <f t="shared" ref="W181" si="162">IF(D181=0,"",$B181)</f>
+        <v/>
+      </c>
+      <c r="Y181" s="1" t="str">
+        <f t="shared" ref="Y181" si="163">IF(E181=0,"",$A181)</f>
+        <v>14.1.0</v>
+      </c>
+      <c r="Z181" s="1" t="str">
+        <f t="shared" ref="Z181" si="164">IF(E181=0,"",$E181)</f>
+        <v>4.0.0</v>
+      </c>
+      <c r="AA181" s="1" t="str">
+        <f t="shared" ref="AA181" si="165">IF(E181=0,"",$B181)</f>
+        <v>14.1.0</v>
+      </c>
+      <c r="AC181" s="1" t="str">
+        <f t="shared" si="65"/>
+        <v/>
+      </c>
+      <c r="AD181" s="1" t="str">
+        <f t="shared" si="66"/>
+        <v/>
+      </c>
+      <c r="AE181" s="1" t="str">
+        <f t="shared" si="67"/>
+        <v/>
+      </c>
+      <c r="AF181" s="1" t="str">
+        <f t="shared" si="68"/>
+        <v/>
+      </c>
+      <c r="AG181" s="1" t="str">
+        <f t="shared" si="69"/>
+        <v/>
+      </c>
+      <c r="AH181" s="1" t="str">
+        <f t="shared" si="70"/>
+        <v/>
+      </c>
+      <c r="AI181" s="1" t="str">
+        <f t="shared" si="71"/>
+        <v/>
+      </c>
+      <c r="AJ181" s="1" t="str">
+        <f t="shared" si="72"/>
+        <v/>
+      </c>
+      <c r="AL181" s="1" t="str">
+        <f t="shared" si="73"/>
+        <v>1.7.0</v>
+      </c>
+      <c r="AM181" s="1" t="str">
+        <f t="shared" si="74"/>
+        <v>14.1.0</v>
+      </c>
+      <c r="AN181" s="1" t="str">
+        <f t="shared" si="75"/>
+        <v>2.0.0</v>
+      </c>
+      <c r="AO181" s="1" t="str">
+        <f t="shared" si="76"/>
+        <v>4.0.0</v>
+      </c>
+      <c r="AP181" s="1" t="str">
+        <f t="shared" si="77"/>
+        <v>7.0.0</v>
+      </c>
+      <c r="AQ181" s="1" t="str">
+        <f t="shared" si="78"/>
+        <v>14.1.0</v>
+      </c>
+      <c r="AR181" s="1" t="str">
+        <f t="shared" si="79"/>
+        <v>3.0.0</v>
+      </c>
+      <c r="AS181" s="1" t="str">
         <f t="shared" si="80"/>
         <v>2.0.0</v>
       </c>
@@ -24938,23 +25223,23 @@
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45">
+      <c r="A45" t="str">
         <f>tables!N180</f>
-        <v>0</v>
-      </c>
-      <c r="B45">
+        <v>14.1.0</v>
+      </c>
+      <c r="B45" t="str">
         <f>tables!O180</f>
-        <v>0</v>
+        <v>14.1.0</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46">
+      <c r="A46" t="str">
         <f>tables!N181</f>
-        <v>0</v>
-      </c>
-      <c r="B46">
+        <v>14.1.0</v>
+      </c>
+      <c r="B46" t="str">
         <f>tables!O181</f>
-        <v>0</v>
+        <v>14.1.0</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -27442,31 +27727,31 @@
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A178">
+      <c r="A178" t="str">
         <f>tables!Q180</f>
-        <v>0</v>
-      </c>
-      <c r="B178">
+        <v/>
+      </c>
+      <c r="B178" t="str">
         <f>tables!R180</f>
-        <v>0</v>
-      </c>
-      <c r="C178">
+        <v/>
+      </c>
+      <c r="C178" t="str">
         <f>tables!S180</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A179">
+      <c r="A179" t="str">
         <f>tables!Q181</f>
-        <v>0</v>
-      </c>
-      <c r="B179">
+        <v/>
+      </c>
+      <c r="B179" t="str">
         <f>tables!R181</f>
-        <v>0</v>
-      </c>
-      <c r="C179">
+        <v/>
+      </c>
+      <c r="C179" t="str">
         <f>tables!S181</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
@@ -30100,43 +30385,43 @@
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="str">
         <f>tables!U179</f>
-        <v/>
+        <v>14.1.0</v>
       </c>
       <c r="B177" t="str">
         <f>tables!V179</f>
-        <v/>
+        <v>10.0.0</v>
       </c>
       <c r="C177" t="str">
         <f>tables!W179</f>
-        <v/>
+        <v>14.1.0</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A178">
+      <c r="A178" t="str">
         <f>tables!U180</f>
-        <v>0</v>
-      </c>
-      <c r="B178">
+        <v/>
+      </c>
+      <c r="B178" t="str">
         <f>tables!V180</f>
-        <v>0</v>
-      </c>
-      <c r="C178">
+        <v/>
+      </c>
+      <c r="C178" t="str">
         <f>tables!W180</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A179">
+      <c r="A179" t="str">
         <f>tables!U181</f>
-        <v>0</v>
-      </c>
-      <c r="B179">
+        <v/>
+      </c>
+      <c r="B179" t="str">
         <f>tables!V181</f>
-        <v>0</v>
-      </c>
-      <c r="C179">
+        <v/>
+      </c>
+      <c r="C179" t="str">
         <f>tables!W181</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
@@ -33350,103 +33635,103 @@
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="str">
         <f>tables!AC179</f>
-        <v/>
+        <v>1.7.0</v>
       </c>
       <c r="B83" t="str">
         <f>tables!AD179</f>
-        <v/>
+        <v>14.1.0</v>
       </c>
       <c r="C83" t="str">
         <f>tables!AE179</f>
-        <v/>
+        <v>9.0.0</v>
       </c>
       <c r="D83" t="str">
         <f>tables!AF179</f>
-        <v/>
+        <v>10.0.0</v>
       </c>
       <c r="E83" t="str">
         <f>tables!AG179</f>
-        <v/>
+        <v>7.0.0</v>
       </c>
       <c r="F83" t="str">
         <f>tables!AH179</f>
-        <v/>
+        <v>14.1.0</v>
       </c>
       <c r="G83" t="str">
         <f>tables!AI179</f>
-        <v/>
+        <v>3.0.0</v>
       </c>
       <c r="H83" t="str">
         <f>tables!AJ179</f>
-        <v/>
+        <v>2.0.0</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A84">
+      <c r="A84" t="str">
         <f>tables!AC180</f>
-        <v>0</v>
-      </c>
-      <c r="B84">
+        <v/>
+      </c>
+      <c r="B84" t="str">
         <f>tables!AD180</f>
-        <v>0</v>
-      </c>
-      <c r="C84">
+        <v/>
+      </c>
+      <c r="C84" t="str">
         <f>tables!AE180</f>
-        <v>0</v>
-      </c>
-      <c r="D84">
+        <v/>
+      </c>
+      <c r="D84" t="str">
         <f>tables!AF180</f>
-        <v>0</v>
-      </c>
-      <c r="E84">
+        <v/>
+      </c>
+      <c r="E84" t="str">
         <f>tables!AG180</f>
-        <v>0</v>
-      </c>
-      <c r="F84">
+        <v/>
+      </c>
+      <c r="F84" t="str">
         <f>tables!AH180</f>
-        <v>0</v>
-      </c>
-      <c r="G84">
+        <v/>
+      </c>
+      <c r="G84" t="str">
         <f>tables!AI180</f>
-        <v>0</v>
-      </c>
-      <c r="H84">
+        <v/>
+      </c>
+      <c r="H84" t="str">
         <f>tables!AJ180</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A85">
+      <c r="A85" t="str">
         <f>tables!AC181</f>
-        <v>0</v>
-      </c>
-      <c r="B85">
+        <v/>
+      </c>
+      <c r="B85" t="str">
         <f>tables!AD181</f>
-        <v>0</v>
-      </c>
-      <c r="C85">
+        <v/>
+      </c>
+      <c r="C85" t="str">
         <f>tables!AE181</f>
-        <v>0</v>
-      </c>
-      <c r="D85">
+        <v/>
+      </c>
+      <c r="D85" t="str">
         <f>tables!AF181</f>
-        <v>0</v>
-      </c>
-      <c r="E85">
+        <v/>
+      </c>
+      <c r="E85" t="str">
         <f>tables!AG181</f>
-        <v>0</v>
-      </c>
-      <c r="F85">
+        <v/>
+      </c>
+      <c r="F85" t="str">
         <f>tables!AH181</f>
-        <v>0</v>
-      </c>
-      <c r="G85">
+        <v/>
+      </c>
+      <c r="G85" t="str">
         <f>tables!AI181</f>
-        <v>0</v>
-      </c>
-      <c r="H85">
+        <v/>
+      </c>
+      <c r="H85" t="str">
         <f>tables!AJ181</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
@@ -42681,103 +42966,103 @@
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f>tables!AL179</f>
-        <v>1.6.0</v>
+        <v/>
       </c>
       <c r="B24" t="str">
         <f>tables!AM179</f>
-        <v>14.1.0</v>
+        <v/>
       </c>
       <c r="C24" t="str">
         <f>tables!AN179</f>
-        <v>2.0.0</v>
+        <v/>
       </c>
       <c r="D24" t="str">
         <f>tables!AO179</f>
-        <v>4.0.0</v>
+        <v/>
       </c>
       <c r="E24" t="str">
         <f>tables!AP179</f>
-        <v>7.0.0</v>
+        <v/>
       </c>
       <c r="F24" t="str">
         <f>tables!AQ179</f>
-        <v>14.1.0</v>
+        <v/>
       </c>
       <c r="G24" t="str">
         <f>tables!AR179</f>
-        <v>3.0.0</v>
+        <v/>
       </c>
       <c r="H24" t="str">
         <f>tables!AS179</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="str">
+        <f>tables!AL180</f>
+        <v>1.6.0</v>
+      </c>
+      <c r="B25" t="str">
+        <f>tables!AM180</f>
+        <v>14.1.0</v>
+      </c>
+      <c r="C25" t="str">
+        <f>tables!AN180</f>
         <v>2.0.0</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <f>tables!AL180</f>
-        <v>0</v>
-      </c>
-      <c r="B25">
-        <f>tables!AM180</f>
-        <v>0</v>
-      </c>
-      <c r="C25">
-        <f>tables!AN180</f>
-        <v>0</v>
-      </c>
-      <c r="D25">
+      <c r="D25" t="str">
         <f>tables!AO180</f>
-        <v>0</v>
-      </c>
-      <c r="E25">
+        <v>4.0.0</v>
+      </c>
+      <c r="E25" t="str">
         <f>tables!AP180</f>
-        <v>0</v>
-      </c>
-      <c r="F25">
+        <v>7.0.0</v>
+      </c>
+      <c r="F25" t="str">
         <f>tables!AQ180</f>
-        <v>0</v>
-      </c>
-      <c r="G25">
+        <v>14.1.0</v>
+      </c>
+      <c r="G25" t="str">
         <f>tables!AR180</f>
-        <v>0</v>
-      </c>
-      <c r="H25">
+        <v>3.0.0</v>
+      </c>
+      <c r="H25" t="str">
         <f>tables!AS180</f>
-        <v>0</v>
+        <v>2.0.0</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26">
+      <c r="A26" t="str">
         <f>tables!AL181</f>
-        <v>0</v>
-      </c>
-      <c r="B26">
+        <v>1.7.0</v>
+      </c>
+      <c r="B26" t="str">
         <f>tables!AM181</f>
-        <v>0</v>
-      </c>
-      <c r="C26">
+        <v>14.1.0</v>
+      </c>
+      <c r="C26" t="str">
         <f>tables!AN181</f>
-        <v>0</v>
-      </c>
-      <c r="D26">
+        <v>2.0.0</v>
+      </c>
+      <c r="D26" t="str">
         <f>tables!AO181</f>
-        <v>0</v>
-      </c>
-      <c r="E26">
+        <v>4.0.0</v>
+      </c>
+      <c r="E26" t="str">
         <f>tables!AP181</f>
-        <v>0</v>
-      </c>
-      <c r="F26">
+        <v>7.0.0</v>
+      </c>
+      <c r="F26" t="str">
         <f>tables!AQ181</f>
-        <v>0</v>
-      </c>
-      <c r="G26">
+        <v>14.1.0</v>
+      </c>
+      <c r="G26" t="str">
         <f>tables!AR181</f>
-        <v>0</v>
-      </c>
-      <c r="H26">
+        <v>3.0.0</v>
+      </c>
+      <c r="H26" t="str">
         <f>tables!AS181</f>
-        <v>0</v>
+        <v>2.0.0</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
replace 14.1.0 by 14.1.1
</commit_message>
<xml_diff>
--- a/VEEPortingGuide/ui_vg_releases_notes_cco.xlsx
+++ b/VEEPortingGuide/ui_vg_releases_notes_cco.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git_pub\docs\VEEPortingGuide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04DC6B09-22D2-4673-9622-B97394F04EC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C8A3FE-A452-4DC0-AB0D-AE341ACC9ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="502" xr2:uid="{62F6EEB7-C17F-40C9-8050-F3352CC93ED9}"/>
   </bookViews>
@@ -307,13 +307,13 @@
     <t>14.0.2</t>
   </si>
   <si>
-    <t>14.1.0</t>
-  </si>
-  <si>
     <t>10.0.0</t>
   </si>
   <si>
     <t>1.7.0</t>
+  </si>
+  <si>
+    <t>14.1.1</t>
   </si>
 </sst>
 </file>
@@ -407,7 +407,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -421,6 +421,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -428,15 +431,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -757,26 +751,26 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:18" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -885,7 +879,7 @@
       <c r="J6" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="K6" s="7" t="s">
         <v>49</v>
       </c>
       <c r="L6" s="1" t="s">
@@ -1028,7 +1022,7 @@
       <c r="D11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="7" t="s">
         <v>31</v>
       </c>
       <c r="H11" s="1" t="s">
@@ -1060,7 +1054,7 @@
       <c r="H12" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="I12" s="11" t="s">
+      <c r="I12" s="7" t="s">
         <v>3</v>
       </c>
       <c r="J12" s="1" t="s">
@@ -1105,15 +1099,15 @@
       <c r="C14" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E14" s="1"/>
+      <c r="H14" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="E14" s="1"/>
-      <c r="H14" s="11" t="s">
-        <v>93</v>
-      </c>
       <c r="I14" s="1"/>
-      <c r="J14" s="11" t="s">
+      <c r="J14" s="7" t="s">
         <v>7</v>
       </c>
       <c r="K14" s="1"/>
@@ -1143,8 +1137,8 @@
       <c r="A16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>91</v>
+      <c r="B16" s="7" t="s">
+        <v>93</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>1</v>
@@ -1163,7 +1157,7 @@
         <v>20</v>
       </c>
       <c r="B17" s="1"/>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="7" t="s">
         <v>3</v>
       </c>
       <c r="D17" s="1"/>
@@ -1277,13 +1271,13 @@
       <c r="M24" s="1"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="1" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A26" s="11" t="s">
-        <v>91</v>
+      <c r="A26" s="7" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1324,65 +1318,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
       <c r="M1" s="4"/>
-      <c r="N1" s="8" t="s">
+      <c r="N1" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="O1" s="8"/>
+      <c r="O1" s="9"/>
       <c r="P1" s="6"/>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="R1" s="8"/>
-      <c r="S1" s="8"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9"/>
       <c r="T1" s="6"/>
-      <c r="U1" s="8" t="s">
+      <c r="U1" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="V1" s="8"/>
-      <c r="W1" s="8"/>
+      <c r="V1" s="9"/>
+      <c r="W1" s="9"/>
       <c r="X1" s="6"/>
-      <c r="Y1" s="8" t="s">
+      <c r="Y1" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="Z1" s="8"/>
-      <c r="AA1" s="8"/>
+      <c r="Z1" s="9"/>
+      <c r="AA1" s="9"/>
       <c r="AB1" s="6"/>
-      <c r="AC1" s="8" t="s">
+      <c r="AC1" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="AD1" s="8"/>
-      <c r="AE1" s="8"/>
-      <c r="AF1" s="8"/>
-      <c r="AG1" s="8"/>
-      <c r="AH1" s="8"/>
-      <c r="AI1" s="8"/>
-      <c r="AJ1" s="8"/>
+      <c r="AD1" s="9"/>
+      <c r="AE1" s="9"/>
+      <c r="AF1" s="9"/>
+      <c r="AG1" s="9"/>
+      <c r="AH1" s="9"/>
+      <c r="AI1" s="9"/>
+      <c r="AJ1" s="9"/>
       <c r="AK1" s="5"/>
-      <c r="AL1" s="8" t="s">
+      <c r="AL1" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="AM1" s="8"/>
-      <c r="AN1" s="8"/>
-      <c r="AO1" s="8"/>
-      <c r="AP1" s="8"/>
-      <c r="AQ1" s="8"/>
-      <c r="AR1" s="8"/>
-      <c r="AS1" s="8"/>
+      <c r="AM1" s="9"/>
+      <c r="AN1" s="9"/>
+      <c r="AO1" s="9"/>
+      <c r="AP1" s="9"/>
+      <c r="AQ1" s="9"/>
+      <c r="AR1" s="9"/>
+      <c r="AS1" s="9"/>
     </row>
     <row r="3" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -23406,11 +23400,11 @@
     </row>
     <row r="172" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A172" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B172" s="3" t="str">
         <f>A172</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C172" s="3"/>
       <c r="D172" s="3"/>
@@ -23423,47 +23417,47 @@
       <c r="K172" s="3"/>
       <c r="L172" s="3"/>
       <c r="N172" s="1" t="str">
-        <f t="shared" ref="N172:N179" si="117">A172</f>
-        <v>14.1.0</v>
+        <f t="shared" ref="N172:N178" si="117">A172</f>
+        <v>14.1.1</v>
       </c>
       <c r="O172" s="1" t="str">
-        <f t="shared" ref="O172:O179" si="118">B172</f>
-        <v>14.1.0</v>
+        <f t="shared" ref="O172:O178" si="118">B172</f>
+        <v>14.1.1</v>
       </c>
       <c r="Q172" s="1" t="str">
-        <f t="shared" ref="Q172:Q179" si="119">IF(C172=0,"",$A172)</f>
+        <f t="shared" ref="Q172:Q178" si="119">IF(C172=0,"",$A172)</f>
         <v/>
       </c>
       <c r="R172" s="1" t="str">
-        <f t="shared" ref="R172:R179" si="120">IF(C172=0,"",$C172)</f>
+        <f t="shared" ref="R172:R178" si="120">IF(C172=0,"",$C172)</f>
         <v/>
       </c>
       <c r="S172" s="1" t="str">
-        <f t="shared" ref="S172:S179" si="121">IF(C172=0,"",$B172)</f>
+        <f t="shared" ref="S172:S178" si="121">IF(C172=0,"",$B172)</f>
         <v/>
       </c>
       <c r="U172" s="1" t="str">
-        <f t="shared" ref="U172:U179" si="122">IF(D172=0,"",$A172)</f>
+        <f t="shared" ref="U172:U178" si="122">IF(D172=0,"",$A172)</f>
         <v/>
       </c>
       <c r="V172" s="1" t="str">
-        <f t="shared" ref="V172:V179" si="123">IF(D172=0,"",$D172)</f>
+        <f t="shared" ref="V172:V178" si="123">IF(D172=0,"",$D172)</f>
         <v/>
       </c>
       <c r="W172" s="1" t="str">
-        <f t="shared" ref="W172:W179" si="124">IF(D172=0,"",$B172)</f>
+        <f t="shared" ref="W172:W178" si="124">IF(D172=0,"",$B172)</f>
         <v/>
       </c>
       <c r="Y172" s="1" t="str">
-        <f t="shared" ref="Y172:Y179" si="125">IF(E172=0,"",$A172)</f>
+        <f t="shared" ref="Y172:Y178" si="125">IF(E172=0,"",$A172)</f>
         <v/>
       </c>
       <c r="Z172" s="1" t="str">
-        <f t="shared" ref="Z172:Z179" si="126">IF(E172=0,"",$E172)</f>
+        <f t="shared" ref="Z172:Z178" si="126">IF(E172=0,"",$E172)</f>
         <v/>
       </c>
       <c r="AA172" s="1" t="str">
-        <f t="shared" ref="AA172:AA179" si="127">IF(E172=0,"",$B172)</f>
+        <f t="shared" ref="AA172:AA178" si="127">IF(E172=0,"",$B172)</f>
         <v/>
       </c>
       <c r="AC172" s="1" t="str">
@@ -23534,11 +23528,11 @@
     <row r="173" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A173" s="3" t="str">
         <f>A172</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B173" s="3" t="str">
         <f t="shared" ref="B173:B181" si="128">A173</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C173" s="3" t="s">
         <v>3</v>
@@ -23554,15 +23548,15 @@
       <c r="L173" s="3"/>
       <c r="N173" s="1" t="str">
         <f t="shared" si="117"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="O173" s="1" t="str">
         <f t="shared" si="118"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Q173" s="1" t="str">
         <f t="shared" si="119"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="R173" s="1" t="str">
         <f t="shared" si="120"/>
@@ -23570,7 +23564,7 @@
       </c>
       <c r="S173" s="1" t="str">
         <f t="shared" si="121"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="U173" s="1" t="str">
         <f t="shared" si="122"/>
@@ -23664,15 +23658,15 @@
     <row r="174" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A174" s="3" t="str">
         <f t="shared" ref="A174:A178" si="129">A173</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B174" s="3" t="str">
         <f t="shared" si="128"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C174" s="3"/>
       <c r="D174" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E174" s="3"/>
       <c r="F174" s="3"/>
@@ -23684,11 +23678,11 @@
       <c r="L174" s="3"/>
       <c r="N174" s="1" t="str">
         <f t="shared" si="117"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="O174" s="1" t="str">
         <f t="shared" si="118"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Q174" s="1" t="str">
         <f t="shared" si="119"/>
@@ -23704,7 +23698,7 @@
       </c>
       <c r="U174" s="1" t="str">
         <f t="shared" si="122"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="V174" s="1" t="str">
         <f t="shared" si="123"/>
@@ -23712,7 +23706,7 @@
       </c>
       <c r="W174" s="1" t="str">
         <f t="shared" si="124"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Y174" s="1" t="str">
         <f t="shared" si="125"/>
@@ -23794,11 +23788,11 @@
     <row r="175" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A175" s="3" t="str">
         <f t="shared" si="129"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B175" s="3" t="str">
         <f t="shared" si="128"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C175" s="3"/>
       <c r="D175" s="3"/>
@@ -23814,11 +23808,11 @@
       <c r="L175" s="3"/>
       <c r="N175" s="1" t="str">
         <f t="shared" si="117"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="O175" s="1" t="str">
         <f t="shared" si="118"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Q175" s="1" t="str">
         <f t="shared" si="119"/>
@@ -23846,7 +23840,7 @@
       </c>
       <c r="Y175" s="1" t="str">
         <f t="shared" si="125"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Z175" s="1" t="str">
         <f t="shared" si="126"/>
@@ -23854,7 +23848,7 @@
       </c>
       <c r="AA175" s="1" t="str">
         <f t="shared" si="127"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AC175" s="1" t="str">
         <f t="shared" si="65"/>
@@ -23924,41 +23918,41 @@
     <row r="176" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A176" s="3" t="str">
         <f t="shared" si="129"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B176" s="3" t="str">
         <f t="shared" si="128"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C176" s="3"/>
-      <c r="D176" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="E176" s="12"/>
-      <c r="F176" s="12"/>
-      <c r="G176" s="12" t="s">
+      <c r="D176" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E176" s="3"/>
+      <c r="F176" s="3"/>
+      <c r="G176" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="H176" s="12" t="s">
+      <c r="H176" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I176" s="12" t="s">
+      <c r="I176" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J176" s="12"/>
-      <c r="K176" s="12" t="s">
+      <c r="J176" s="3"/>
+      <c r="K176" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="L176" s="12" t="s">
+      <c r="L176" s="3" t="s">
         <v>49</v>
       </c>
       <c r="N176" s="1" t="str">
         <f t="shared" si="117"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="O176" s="1" t="str">
         <f t="shared" si="118"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Q176" s="1" t="str">
         <f t="shared" si="119"/>
@@ -23974,7 +23968,7 @@
       </c>
       <c r="U176" s="1" t="str">
         <f t="shared" si="122"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="V176" s="1" t="str">
         <f t="shared" si="123"/>
@@ -23982,7 +23976,7 @@
       </c>
       <c r="W176" s="1" t="str">
         <f t="shared" si="124"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Y176" s="1" t="str">
         <f t="shared" si="125"/>
@@ -24002,7 +23996,7 @@
       </c>
       <c r="AD176" s="1" t="str">
         <f t="shared" si="66"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AE176" s="1" t="str">
         <f t="shared" si="67"/>
@@ -24018,7 +24012,7 @@
       </c>
       <c r="AH176" s="1" t="str">
         <f t="shared" si="70"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AI176" s="1" t="str">
         <f t="shared" si="71"/>
@@ -24064,41 +24058,41 @@
     <row r="177" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A177" s="3" t="str">
         <f t="shared" si="129"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B177" s="3" t="str">
         <f t="shared" si="128"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C177" s="3"/>
-      <c r="D177" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="E177" s="12"/>
-      <c r="F177" s="12"/>
-      <c r="G177" s="12" t="s">
+      <c r="D177" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E177" s="3"/>
+      <c r="F177" s="3"/>
+      <c r="G177" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="H177" s="12" t="s">
+      <c r="H177" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I177" s="12" t="s">
+      <c r="I177" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J177" s="12"/>
-      <c r="K177" s="12" t="s">
+      <c r="J177" s="3"/>
+      <c r="K177" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="L177" s="12" t="s">
+      <c r="L177" s="3" t="s">
         <v>49</v>
       </c>
       <c r="N177" s="1" t="str">
         <f t="shared" si="117"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="O177" s="1" t="str">
         <f t="shared" si="118"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Q177" s="1" t="str">
         <f t="shared" si="119"/>
@@ -24114,7 +24108,7 @@
       </c>
       <c r="U177" s="1" t="str">
         <f t="shared" si="122"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="V177" s="1" t="str">
         <f t="shared" si="123"/>
@@ -24122,7 +24116,7 @@
       </c>
       <c r="W177" s="1" t="str">
         <f t="shared" si="124"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Y177" s="1" t="str">
         <f t="shared" si="125"/>
@@ -24142,7 +24136,7 @@
       </c>
       <c r="AD177" s="1" t="str">
         <f t="shared" si="66"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AE177" s="1" t="str">
         <f t="shared" si="67"/>
@@ -24158,7 +24152,7 @@
       </c>
       <c r="AH177" s="1" t="str">
         <f t="shared" si="70"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AI177" s="1" t="str">
         <f t="shared" si="71"/>
@@ -24204,41 +24198,41 @@
     <row r="178" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A178" s="3" t="str">
         <f t="shared" si="129"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B178" s="3" t="str">
         <f t="shared" si="128"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C178" s="3"/>
-      <c r="D178" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="E178" s="12"/>
-      <c r="F178" s="12"/>
-      <c r="G178" s="12" t="s">
+      <c r="D178" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E178" s="3"/>
+      <c r="F178" s="3"/>
+      <c r="G178" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="H178" s="12" t="s">
+      <c r="H178" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I178" s="12" t="s">
+      <c r="I178" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J178" s="12"/>
-      <c r="K178" s="12" t="s">
+      <c r="J178" s="3"/>
+      <c r="K178" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="L178" s="12" t="s">
+      <c r="L178" s="3" t="s">
         <v>49</v>
       </c>
       <c r="N178" s="1" t="str">
         <f t="shared" si="117"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="O178" s="1" t="str">
         <f t="shared" si="118"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Q178" s="1" t="str">
         <f t="shared" si="119"/>
@@ -24254,7 +24248,7 @@
       </c>
       <c r="U178" s="1" t="str">
         <f t="shared" si="122"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="V178" s="1" t="str">
         <f t="shared" si="123"/>
@@ -24262,7 +24256,7 @@
       </c>
       <c r="W178" s="1" t="str">
         <f t="shared" si="124"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Y178" s="1" t="str">
         <f t="shared" si="125"/>
@@ -24282,7 +24276,7 @@
       </c>
       <c r="AD178" s="1" t="str">
         <f t="shared" si="66"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AE178" s="1" t="str">
         <f t="shared" si="67"/>
@@ -24298,7 +24292,7 @@
       </c>
       <c r="AH178" s="1" t="str">
         <f t="shared" si="70"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AI178" s="1" t="str">
         <f t="shared" si="71"/>
@@ -24344,41 +24338,41 @@
     <row r="179" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A179" s="3" t="str">
         <f t="shared" ref="A179" si="130">A178</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B179" s="3" t="str">
         <f t="shared" si="128"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C179" s="3"/>
-      <c r="D179" s="12" t="s">
+      <c r="D179" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E179" s="3"/>
+      <c r="F179" s="3"/>
+      <c r="G179" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E179" s="12"/>
-      <c r="F179" s="12"/>
-      <c r="G179" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="H179" s="12" t="s">
+      <c r="H179" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I179" s="12" t="s">
+      <c r="I179" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J179" s="12"/>
-      <c r="K179" s="12" t="s">
+      <c r="J179" s="3"/>
+      <c r="K179" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="L179" s="12" t="s">
+      <c r="L179" s="3" t="s">
         <v>49</v>
       </c>
       <c r="N179" s="1" t="str">
         <f t="shared" ref="N179" si="131">A179</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="O179" s="1" t="str">
         <f t="shared" ref="O179" si="132">B179</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Q179" s="1" t="str">
         <f t="shared" ref="Q179" si="133">IF(C179=0,"",$A179)</f>
@@ -24394,7 +24388,7 @@
       </c>
       <c r="U179" s="1" t="str">
         <f t="shared" ref="U179" si="136">IF(D179=0,"",$A179)</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="V179" s="1" t="str">
         <f t="shared" ref="V179" si="137">IF(D179=0,"",$D179)</f>
@@ -24402,7 +24396,7 @@
       </c>
       <c r="W179" s="1" t="str">
         <f t="shared" ref="W179" si="138">IF(D179=0,"",$B179)</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Y179" s="1" t="str">
         <f t="shared" ref="Y179" si="139">IF(E179=0,"",$A179)</f>
@@ -24422,7 +24416,7 @@
       </c>
       <c r="AD179" s="1" t="str">
         <f t="shared" si="66"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AE179" s="1" t="str">
         <f t="shared" si="67"/>
@@ -24438,7 +24432,7 @@
       </c>
       <c r="AH179" s="1" t="str">
         <f t="shared" si="70"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AI179" s="1" t="str">
         <f t="shared" si="71"/>
@@ -24484,41 +24478,41 @@
     <row r="180" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A180" s="3" t="str">
         <f t="shared" ref="A180" si="142">A179</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B180" s="3" t="str">
         <f t="shared" si="128"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C180" s="3"/>
-      <c r="D180" s="12"/>
-      <c r="E180" s="12" t="s">
+      <c r="D180" s="3"/>
+      <c r="E180" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F180" s="12"/>
-      <c r="G180" s="12" t="s">
+      <c r="F180" s="3"/>
+      <c r="G180" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="H180" s="12" t="s">
+      <c r="H180" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I180" s="12"/>
-      <c r="J180" s="12" t="s">
+      <c r="I180" s="3"/>
+      <c r="J180" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="K180" s="12" t="s">
+      <c r="K180" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="L180" s="12" t="s">
+      <c r="L180" s="3" t="s">
         <v>49</v>
       </c>
       <c r="N180" s="1" t="str">
         <f t="shared" ref="N180" si="143">A180</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="O180" s="1" t="str">
         <f t="shared" ref="O180" si="144">B180</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Q180" s="1" t="str">
         <f t="shared" ref="Q180" si="145">IF(C180=0,"",$A180)</f>
@@ -24546,7 +24540,7 @@
       </c>
       <c r="Y180" s="1" t="str">
         <f t="shared" ref="Y180" si="151">IF(E180=0,"",$A180)</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Z180" s="1" t="str">
         <f t="shared" ref="Z180" si="152">IF(E180=0,"",$E180)</f>
@@ -24554,7 +24548,7 @@
       </c>
       <c r="AA180" s="1" t="str">
         <f t="shared" ref="AA180" si="153">IF(E180=0,"",$B180)</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AC180" s="1" t="str">
         <f t="shared" si="65"/>
@@ -24594,7 +24588,7 @@
       </c>
       <c r="AM180" s="1" t="str">
         <f t="shared" si="74"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AN180" s="1" t="str">
         <f t="shared" si="75"/>
@@ -24610,7 +24604,7 @@
       </c>
       <c r="AQ180" s="1" t="str">
         <f t="shared" si="78"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AR180" s="1" t="str">
         <f t="shared" si="79"/>
@@ -24624,41 +24618,41 @@
     <row r="181" spans="1:45" x14ac:dyDescent="0.25">
       <c r="A181" s="3" t="str">
         <f t="shared" ref="A181" si="154">A180</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B181" s="3" t="str">
         <f t="shared" si="128"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C181" s="3"/>
-      <c r="D181" s="12"/>
-      <c r="E181" s="12" t="s">
+      <c r="D181" s="3"/>
+      <c r="E181" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F181" s="12"/>
-      <c r="G181" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="H181" s="12" t="s">
+      <c r="F181" s="3"/>
+      <c r="G181" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H181" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I181" s="12"/>
-      <c r="J181" s="12" t="s">
+      <c r="I181" s="3"/>
+      <c r="J181" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="K181" s="12" t="s">
+      <c r="K181" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="L181" s="12" t="s">
+      <c r="L181" s="3" t="s">
         <v>49</v>
       </c>
       <c r="N181" s="1" t="str">
         <f t="shared" ref="N181" si="155">A181</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="O181" s="1" t="str">
         <f t="shared" ref="O181" si="156">B181</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Q181" s="1" t="str">
         <f t="shared" ref="Q181" si="157">IF(C181=0,"",$A181)</f>
@@ -24686,7 +24680,7 @@
       </c>
       <c r="Y181" s="1" t="str">
         <f t="shared" ref="Y181" si="163">IF(E181=0,"",$A181)</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="Z181" s="1" t="str">
         <f t="shared" ref="Z181" si="164">IF(E181=0,"",$E181)</f>
@@ -24694,7 +24688,7 @@
       </c>
       <c r="AA181" s="1" t="str">
         <f t="shared" ref="AA181" si="165">IF(E181=0,"",$B181)</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AC181" s="1" t="str">
         <f t="shared" si="65"/>
@@ -24734,7 +24728,7 @@
       </c>
       <c r="AM181" s="1" t="str">
         <f t="shared" si="74"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AN181" s="1" t="str">
         <f t="shared" si="75"/>
@@ -24750,7 +24744,7 @@
       </c>
       <c r="AQ181" s="1" t="str">
         <f t="shared" si="78"/>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="AR181" s="1" t="str">
         <f t="shared" si="79"/>
@@ -25145,101 +25139,101 @@
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
         <f>tables!N172</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B37" t="str">
         <f>tables!O172</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
         <f>tables!N173</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B38" t="str">
         <f>tables!O173</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
         <f>tables!N174</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B39" t="str">
         <f>tables!O174</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
         <f>tables!N175</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B40" t="str">
         <f>tables!O175</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="str">
         <f>tables!N176</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B41" t="str">
         <f>tables!O176</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="str">
         <f>tables!N177</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B42" t="str">
         <f>tables!O177</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="str">
         <f>tables!N178</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B43" t="str">
         <f>tables!O178</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="str">
         <f>tables!N179</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B44" t="str">
         <f>tables!O179</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="str">
         <f>tables!N180</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B45" t="str">
         <f>tables!O180</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
         <f>tables!N181</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B46" t="str">
         <f>tables!O181</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -27631,7 +27625,7 @@
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="str">
         <f>tables!Q173</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B171" t="str">
         <f>tables!R173</f>
@@ -27639,7 +27633,7 @@
       </c>
       <c r="C171" t="str">
         <f>tables!S173</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
@@ -30315,7 +30309,7 @@
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="str">
         <f>tables!U174</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B172" t="str">
         <f>tables!V174</f>
@@ -30323,7 +30317,7 @@
       </c>
       <c r="C172" t="str">
         <f>tables!W174</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
@@ -30343,7 +30337,7 @@
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="str">
         <f>tables!U176</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B174" t="str">
         <f>tables!V176</f>
@@ -30351,13 +30345,13 @@
       </c>
       <c r="C174" t="str">
         <f>tables!W176</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="str">
         <f>tables!U177</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B175" t="str">
         <f>tables!V177</f>
@@ -30365,13 +30359,13 @@
       </c>
       <c r="C175" t="str">
         <f>tables!W177</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="str">
         <f>tables!U178</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B176" t="str">
         <f>tables!V178</f>
@@ -30379,13 +30373,13 @@
       </c>
       <c r="C176" t="str">
         <f>tables!W178</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="str">
         <f>tables!U179</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B177" t="str">
         <f>tables!V179</f>
@@ -30393,7 +30387,7 @@
       </c>
       <c r="C177" t="str">
         <f>tables!W179</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
@@ -30941,7 +30935,7 @@
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f>tables!Y175</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="B33" t="str">
         <f>tables!Z175</f>
@@ -30949,7 +30943,7 @@
       </c>
       <c r="C33" t="str">
         <f>tables!AA175</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -33163,7 +33157,7 @@
       </c>
       <c r="B69" t="str">
         <f>tables!AD176</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C69" t="str">
         <f>tables!AE176</f>
@@ -33179,7 +33173,7 @@
       </c>
       <c r="F69" t="str">
         <f>tables!AH176</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="G69" t="str">
         <f>tables!AI176</f>
@@ -33197,7 +33191,7 @@
       </c>
       <c r="B70" t="str">
         <f>tables!AD177</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C70" t="str">
         <f>tables!AE177</f>
@@ -33213,7 +33207,7 @@
       </c>
       <c r="F70" t="str">
         <f>tables!AH177</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="G70" t="str">
         <f>tables!AI177</f>
@@ -33537,7 +33531,7 @@
       </c>
       <c r="B80" t="str">
         <f>tables!AD176</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C80" t="str">
         <f>tables!AE176</f>
@@ -33553,7 +33547,7 @@
       </c>
       <c r="F80" t="str">
         <f>tables!AH176</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="G80" t="str">
         <f>tables!AI176</f>
@@ -33571,7 +33565,7 @@
       </c>
       <c r="B81" t="str">
         <f>tables!AD177</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C81" t="str">
         <f>tables!AE177</f>
@@ -33587,7 +33581,7 @@
       </c>
       <c r="F81" t="str">
         <f>tables!AH177</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="G81" t="str">
         <f>tables!AI177</f>
@@ -33605,7 +33599,7 @@
       </c>
       <c r="B82" t="str">
         <f>tables!AD178</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C82" t="str">
         <f>tables!AE178</f>
@@ -33621,7 +33615,7 @@
       </c>
       <c r="F82" t="str">
         <f>tables!AH178</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="G82" t="str">
         <f>tables!AI178</f>
@@ -33639,7 +33633,7 @@
       </c>
       <c r="B83" t="str">
         <f>tables!AD179</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C83" t="str">
         <f>tables!AE179</f>
@@ -33655,7 +33649,7 @@
       </c>
       <c r="F83" t="str">
         <f>tables!AH179</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="G83" t="str">
         <f>tables!AI179</f>
@@ -43004,7 +42998,7 @@
       </c>
       <c r="B25" t="str">
         <f>tables!AM180</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C25" t="str">
         <f>tables!AN180</f>
@@ -43020,7 +43014,7 @@
       </c>
       <c r="F25" t="str">
         <f>tables!AQ180</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="G25" t="str">
         <f>tables!AR180</f>
@@ -43038,7 +43032,7 @@
       </c>
       <c r="B26" t="str">
         <f>tables!AM181</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="C26" t="str">
         <f>tables!AN181</f>
@@ -43054,7 +43048,7 @@
       </c>
       <c r="F26" t="str">
         <f>tables!AQ181</f>
-        <v>14.1.0</v>
+        <v>14.1.1</v>
       </c>
       <c r="G26" t="str">
         <f>tables!AR181</f>

</xml_diff>